<commit_message>
Move tables and send/busy-hour rules into the survey
Ask the table list (new 卓 section) and the send-fare and busy-hour
wage rules (pay section, behind yes/no questions) in the survey as
row tables, and drop those two themes from the LINE/Excel templates so
stores are not asked twice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7QD3LQaBHevrAWkRrJmwD
</commit_message>
<xml_diff>
--- a/templates/excel/初期設定_記入シート.xlsx
+++ b/templates/excel/初期設定_記入シート.xlsx
@@ -10,9 +10,7 @@
     <sheet name="料金セット" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="指名区分" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="商品メニュー" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="卓" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="名簿" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="送り・繁忙" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="名簿" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1909,209 +1907,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>卓</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>※灰色の行は記入例です。消して上書きするか、下の空欄に書いてください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>※配置は、訪問時にPOSの画面で一緒に決めます</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>卓の一覧</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>卓名</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>席数(任意)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>VIP1</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>カウンター</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="6" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="6" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="6" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B9:B38" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2523,392 +2318,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C71"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>送り・繁忙時間帯</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>※灰色の行は記入例です。消して上書きするか、下の空欄に書いてください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>送りエリアごとの送り代</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>エリア名</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>送り代(円)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>みなとみらい</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>関内</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="6" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="6" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="6" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="6" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>時給を上げる時間帯(ある場合のみ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>開始</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>終了</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>倍率または加算額</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>24:00</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>1.2倍</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="6" t="n"/>
-      <c r="C42" s="6" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="6" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="6" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="6" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="n"/>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="6" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="6" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="6" t="n"/>
-      <c r="C49" s="6" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="6" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="6" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="6" t="n"/>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="6" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="6" t="n"/>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="n"/>
-      <c r="B54" s="6" t="n"/>
-      <c r="C54" s="6" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="n"/>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="6" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="6" t="n"/>
-      <c r="B56" s="6" t="n"/>
-      <c r="C56" s="6" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="n"/>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="6" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="6" t="n"/>
-      <c r="B58" s="6" t="n"/>
-      <c r="C58" s="6" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="6" t="n"/>
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="6" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="6" t="n"/>
-      <c r="B60" s="6" t="n"/>
-      <c r="C60" s="6" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="6" t="n"/>
-      <c r="B61" s="6" t="n"/>
-      <c r="C61" s="6" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="6" t="n"/>
-      <c r="B62" s="6" t="n"/>
-      <c r="C62" s="6" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="6" t="n"/>
-      <c r="B63" s="6" t="n"/>
-      <c r="C63" s="6" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="n"/>
-      <c r="B64" s="6" t="n"/>
-      <c r="C64" s="6" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="6" t="n"/>
-      <c r="B65" s="6" t="n"/>
-      <c r="C65" s="6" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="6" t="n"/>
-      <c r="B66" s="6" t="n"/>
-      <c r="C66" s="6" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="6" t="n"/>
-      <c r="B67" s="6" t="n"/>
-      <c r="C67" s="6" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="6" t="n"/>
-      <c r="B68" s="6" t="n"/>
-      <c r="C68" s="6" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="6" t="n"/>
-      <c r="B69" s="6" t="n"/>
-      <c r="C69" s="6" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="6" t="n"/>
-      <c r="B70" s="6" t="n"/>
-      <c r="C70" s="6" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="6" t="n"/>
-      <c r="B71" s="6" t="n"/>
-      <c r="C71" s="6" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B8:B37" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Change the nomination charge unit to minutes
Replace the per-visit/per-hour dropdown with a number of minutes in
the nomination template (LINE, Excel, Google Sheets).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7QD3LQaBHevrAWkRrJmwD
</commit_message>
<xml_diff>
--- a/templates/excel/初期設定_記入シート.xlsx
+++ b/templates/excel/初期設定_記入シート.xlsx
@@ -1056,7 +1056,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>課金単位</t>
+          <t>課金単位(何分ごと)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1118,10 +1118,8 @@
       <c r="B6" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>1接客ごと</t>
-        </is>
+      <c r="C6" s="5" t="n">
+        <v>60</v>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
@@ -1141,10 +1139,8 @@
       <c r="B7" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>1接客ごと</t>
-        </is>
+      <c r="C7" s="5" t="n">
+        <v>60</v>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
@@ -1164,10 +1160,8 @@
       <c r="B8" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>1接客ごと</t>
-        </is>
+      <c r="C8" s="5" t="n">
+        <v>60</v>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
@@ -1187,11 +1181,7 @@
       <c r="B9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>1接客ごと</t>
-        </is>
-      </c>
+      <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>なし</t>
@@ -1414,8 +1404,8 @@
     <dataValidation sqref="B10:B39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="C10:C39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
-      <formula1>"1接客ごと,1時間ごと"</formula1>
+    <dataValidation sqref="C10:C39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="D10:D39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
       <formula1>"円,%,なし"</formula1>

</xml_diff>

<commit_message>
Drop redundant columns from the price set and product sheets
Remove the extension fee column from sets (the extension menu below
lists it), the show-on-floor column from the extension menu, and the
cost and tax columns from products. Point to the regenerated Google
spreadsheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7QD3LQaBHevrAWkRrJmwD
</commit_message>
<xml_diff>
--- a/templates/excel/初期設定_記入シート.xlsx
+++ b/templates/excel/初期設定_記入シート.xlsx
@@ -468,14 +468,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,11 +534,6 @@
           <t>延長(分)</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>延長料金(円)</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -556,9 +550,6 @@
       <c r="D8" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>4000</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -574,9 +565,6 @@
       </c>
       <c r="D9" s="6" t="n">
         <v>30</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>8000</v>
       </c>
     </row>
     <row r="10">
@@ -584,210 +572,180 @@
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
       <c r="B14" s="7" t="n"/>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
       <c r="B23" s="7" t="n"/>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
       <c r="B25" s="7" t="n"/>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
       <c r="B31" s="7" t="n"/>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
       <c r="B32" s="7" t="n"/>
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
       <c r="B33" s="7" t="n"/>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
       <c r="B34" s="7" t="n"/>
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
       <c r="B36" s="7" t="n"/>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
       <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
       <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
       <c r="B39" s="7" t="n"/>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -812,11 +770,6 @@
           <t>料金(円)</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>現場に出す</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -830,11 +783,6 @@
       <c r="C43" s="6" t="n">
         <v>4000</v>
       </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -847,195 +795,160 @@
       </c>
       <c r="C44" s="6" t="n">
         <v>8000</v>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n"/>
       <c r="B45" s="7" t="n"/>
       <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n"/>
       <c r="B46" s="7" t="n"/>
       <c r="C46" s="7" t="n"/>
-      <c r="D46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n"/>
       <c r="B47" s="7" t="n"/>
       <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
       <c r="B48" s="7" t="n"/>
       <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n"/>
       <c r="B49" s="7" t="n"/>
       <c r="C49" s="7" t="n"/>
-      <c r="D49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n"/>
       <c r="B50" s="7" t="n"/>
       <c r="C50" s="7" t="n"/>
-      <c r="D50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
       <c r="B51" s="7" t="n"/>
       <c r="C51" s="7" t="n"/>
-      <c r="D51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
       <c r="B52" s="7" t="n"/>
       <c r="C52" s="7" t="n"/>
-      <c r="D52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n"/>
       <c r="B53" s="7" t="n"/>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
       <c r="B54" s="7" t="n"/>
       <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
       <c r="B55" s="7" t="n"/>
       <c r="C55" s="7" t="n"/>
-      <c r="D55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
       <c r="B56" s="7" t="n"/>
       <c r="C56" s="7" t="n"/>
-      <c r="D56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
       <c r="B57" s="7" t="n"/>
       <c r="C57" s="7" t="n"/>
-      <c r="D57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
       <c r="B58" s="7" t="n"/>
       <c r="C58" s="7" t="n"/>
-      <c r="D58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
       <c r="B59" s="7" t="n"/>
       <c r="C59" s="7" t="n"/>
-      <c r="D59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n"/>
       <c r="B60" s="7" t="n"/>
       <c r="C60" s="7" t="n"/>
-      <c r="D60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="n"/>
       <c r="B61" s="7" t="n"/>
       <c r="C61" s="7" t="n"/>
-      <c r="D61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n"/>
       <c r="B62" s="7" t="n"/>
       <c r="C62" s="7" t="n"/>
-      <c r="D62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n"/>
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="7" t="n"/>
-      <c r="D63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n"/>
       <c r="B64" s="7" t="n"/>
       <c r="C64" s="7" t="n"/>
-      <c r="D64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n"/>
       <c r="B65" s="7" t="n"/>
       <c r="C65" s="7" t="n"/>
-      <c r="D65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n"/>
       <c r="B66" s="7" t="n"/>
       <c r="C66" s="7" t="n"/>
-      <c r="D66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n"/>
       <c r="B67" s="7" t="n"/>
       <c r="C67" s="7" t="n"/>
-      <c r="D67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n"/>
       <c r="B68" s="7" t="n"/>
       <c r="C68" s="7" t="n"/>
-      <c r="D68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n"/>
       <c r="B69" s="7" t="n"/>
       <c r="C69" s="7" t="n"/>
-      <c r="D69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n"/>
       <c r="B70" s="7" t="n"/>
       <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n"/>
       <c r="B71" s="7" t="n"/>
       <c r="C71" s="7" t="n"/>
-      <c r="D71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n"/>
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="7" t="n"/>
-      <c r="D72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="n"/>
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="7" t="n"/>
-      <c r="D73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n"/>
       <c r="B74" s="7" t="n"/>
       <c r="C74" s="7" t="n"/>
-      <c r="D74" s="7" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="5">
     <dataValidation sqref="B10:B39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
@@ -1045,17 +958,11 @@
     <dataValidation sqref="D10:D39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="E10:E39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
     <dataValidation sqref="B45:B74" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="C45:C74" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="D45:D74" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
-      <formula1>"○,×"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1456,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1464,9 +1371,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1528,22 +1433,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>原価(円・任意)</t>
+          <t>キャストドリンク</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>キャストドリンク</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
           <t>ボトルキープ</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>税区分</t>
         </is>
       </c>
     </row>
@@ -1566,18 +1461,10 @@
       <c r="D8" s="6" t="n">
         <v>28000</v>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>○</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>標準10%</t>
         </is>
       </c>
     </row>
@@ -1600,18 +1487,12 @@
       <c r="D9" s="6" t="n">
         <v>800</v>
       </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>標準10%</t>
-        </is>
-      </c>
+      <c r="F9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -1620,8 +1501,6 @@
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -1630,8 +1509,6 @@
       <c r="D11" s="7" t="n"/>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1640,8 +1517,6 @@
       <c r="D12" s="7" t="n"/>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -1650,8 +1525,6 @@
       <c r="D13" s="7" t="n"/>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1660,8 +1533,6 @@
       <c r="D14" s="7" t="n"/>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1670,8 +1541,6 @@
       <c r="D15" s="7" t="n"/>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1680,8 +1549,6 @@
       <c r="D16" s="7" t="n"/>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1690,8 +1557,6 @@
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1700,8 +1565,6 @@
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -1710,8 +1573,6 @@
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -1720,8 +1581,6 @@
       <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -1730,8 +1589,6 @@
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -1740,8 +1597,6 @@
       <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -1750,8 +1605,6 @@
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -1760,8 +1613,6 @@
       <c r="D24" s="7" t="n"/>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -1770,8 +1621,6 @@
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -1780,8 +1629,6 @@
       <c r="D26" s="7" t="n"/>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="7" t="n"/>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -1790,8 +1637,6 @@
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="7" t="n"/>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -1800,8 +1645,6 @@
       <c r="D28" s="7" t="n"/>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
-      <c r="H28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -1810,8 +1653,6 @@
       <c r="D29" s="7" t="n"/>
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="7" t="n"/>
-      <c r="G29" s="7" t="n"/>
-      <c r="H29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -1820,8 +1661,6 @@
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="7" t="n"/>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -1830,8 +1669,6 @@
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -1840,8 +1677,6 @@
       <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="7" t="n"/>
-      <c r="G32" s="7" t="n"/>
-      <c r="H32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -1850,8 +1685,6 @@
       <c r="D33" s="7" t="n"/>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="7" t="n"/>
-      <c r="G33" s="7" t="n"/>
-      <c r="H33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -1860,8 +1693,6 @@
       <c r="D34" s="7" t="n"/>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="7" t="n"/>
-      <c r="G34" s="7" t="n"/>
-      <c r="H34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -1870,8 +1701,6 @@
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="7" t="n"/>
-      <c r="G35" s="7" t="n"/>
-      <c r="H35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -1880,8 +1709,6 @@
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="7" t="n"/>
-      <c r="G36" s="7" t="n"/>
-      <c r="H36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -1890,8 +1717,6 @@
       <c r="D37" s="7" t="n"/>
       <c r="E37" s="7" t="n"/>
       <c r="F37" s="7" t="n"/>
-      <c r="G37" s="7" t="n"/>
-      <c r="H37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -1900,8 +1725,6 @@
       <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
       <c r="F38" s="7" t="n"/>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -1910,28 +1733,20 @@
       <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="7" t="n"/>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="7" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="4">
     <dataValidation sqref="B10:B39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
       <formula1>"ドリンク,ボトル,フード,その他"</formula1>
     </dataValidation>
     <dataValidation sqref="D10:D39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="E10:E39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
+    <dataValidation sqref="E10:E39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
+      <formula1>"○"</formula1>
     </dataValidation>
     <dataValidation sqref="F10:F39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
       <formula1>"○"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G10:G39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
-      <formula1>"○"</formula1>
-    </dataValidation>
-    <dataValidation sqref="H10:H39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
-      <formula1>"標準10%,軽減8%"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Explain cast drinks and their back at the top of the product menu sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7QD3LQaBHevrAWkRrJmwD
</commit_message>
<xml_diff>
--- a/templates/excel/初期設定_記入シート.xlsx
+++ b/templates/excel/初期設定_記入シート.xlsx
@@ -1363,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1399,132 +1399,128 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
+          <t>※「キャストドリンク」は、お客様がキャストにごちそうするドリンクです</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>※○を付けた商品は、注文が入るとキャストにバックが付きます</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>※例)800円のウーロン茶なら、その○%がキャストのバックになります</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>※バックの%や金額はキャストごとに違うので、訪問時に一緒に決めます</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
           <t>※書き終わったら、このファイル(またはシートのリンク)をLINEで送ってください。</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>商品</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>カテゴリー</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>種別</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>商品名</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>価格(円)</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>キャストドリンク</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>ボトルキープ</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>シャンパン</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>ボトル</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>ヴーヴクリコ</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D12" s="6" t="n">
         <v>28000</v>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>ソフトドリンク</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>ドリンク</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>ウーロン茶</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D13" s="6" t="n">
         <v>800</v>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
+      <c r="F13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1734,18 +1730,50 @@
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="7" t="n"/>
     </row>
+    <row r="40">
+      <c r="A40" s="7" t="n"/>
+      <c r="B40" s="7" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="7" t="n"/>
+      <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="n"/>
+      <c r="B41" s="7" t="n"/>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="n"/>
+      <c r="B42" s="7" t="n"/>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="7" t="n"/>
+      <c r="E42" s="7" t="n"/>
+      <c r="F42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="n"/>
+      <c r="B43" s="7" t="n"/>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="7" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="B10:B39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
+    <dataValidation sqref="B14:B43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
       <formula1>"ドリンク,ボトル,フード,その他"</formula1>
     </dataValidation>
-    <dataValidation sqref="D10:D39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="D14:D43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="E10:E39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
+    <dataValidation sqref="E14:E43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
       <formula1>"○"</formula1>
     </dataValidation>
-    <dataValidation sqref="F10:F39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
+    <dataValidation sqref="F14:F43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
       <formula1>"○"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Ask about every back rule the POS supports in section 4
Adds store-wide sales, food back, bottle split, help back and the
closing-time rules (sliding scale, count bonus), matching the rule types
in ポッキリ.Night. The nomination sheet gets the per-visit or per-hour unit
for yen backs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7QD3LQaBHevrAWkRrJmwD
</commit_message>
<xml_diff>
--- a/templates/excel/初期設定_記入シート.xlsx
+++ b/templates/excel/初期設定_記入シート.xlsx
@@ -975,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -983,6 +983,7 @@
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1047,6 +1048,11 @@
           <t>金額または率</t>
         </is>
       </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>円のときの単位</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -1068,6 +1074,11 @@
       <c r="E8" s="6" t="n">
         <v>1000</v>
       </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>1接客ごと</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1089,6 +1100,7 @@
       <c r="E9" s="6" t="n">
         <v>50</v>
       </c>
+      <c r="F9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -1110,6 +1122,11 @@
       <c r="E10" s="6" t="n">
         <v>1000</v>
       </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>1接客ごと</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1127,6 +1144,7 @@
         </is>
       </c>
       <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1134,6 +1152,7 @@
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
       <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -1141,6 +1160,7 @@
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
       <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1148,6 +1168,7 @@
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
       <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -1155,6 +1176,7 @@
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
       <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -1162,6 +1184,7 @@
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
       <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1169,6 +1192,7 @@
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1176,6 +1200,7 @@
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
       <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -1183,6 +1208,7 @@
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -1190,6 +1216,7 @@
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -1197,6 +1224,7 @@
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -1204,6 +1232,7 @@
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -1211,6 +1240,7 @@
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -1218,6 +1248,7 @@
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
       <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -1225,6 +1256,7 @@
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -1232,6 +1264,7 @@
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
       <c r="E26" s="7" t="n"/>
+      <c r="F26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -1239,6 +1272,7 @@
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -1246,6 +1280,7 @@
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="7" t="n"/>
       <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -1253,6 +1288,7 @@
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="7" t="n"/>
       <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -1260,6 +1296,7 @@
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -1267,6 +1304,7 @@
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -1274,6 +1312,7 @@
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="7" t="n"/>
       <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -1281,6 +1320,7 @@
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="n"/>
       <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -1288,6 +1328,7 @@
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="n"/>
       <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -1295,6 +1336,7 @@
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="n"/>
+      <c r="F35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -1302,6 +1344,7 @@
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -1309,6 +1352,7 @@
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
       <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -1316,6 +1360,7 @@
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
+      <c r="F38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -1323,6 +1368,7 @@
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -1330,6 +1376,7 @@
       <c r="C40" s="7" t="n"/>
       <c r="D40" s="7" t="n"/>
       <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -1337,9 +1384,10 @@
       <c r="C41" s="7" t="n"/>
       <c r="D41" s="7" t="n"/>
       <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="B12:B41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
@@ -1351,6 +1399,9 @@
     </dataValidation>
     <dataValidation sqref="E12:E41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="0以上の数字で入力してください" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="F12:F41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
+      <formula1>"1接客ごと,1時間ごと"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Move nomination types into the survey and ask about extension back
The nomination table (fee, interval, back in yen or % and its unit) is
now filled in on section 4, so the LINE/Excel kit drops its sheet.
Extension back gets the same store-wide or per-cast choice as the others.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7QD3LQaBHevrAWkRrJmwD
</commit_message>
<xml_diff>
--- a/templates/excel/初期設定_記入シート.xlsx
+++ b/templates/excel/初期設定_記入シート.xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="料金セット" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="指名区分" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="商品メニュー" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="名簿" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="商品メニュー" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="名簿" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -975,445 +974,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>指名区分</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>店舗名</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>※灰色の行は記入例です。消して上書きするか、下の空欄に書いてください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>※書き終わったら、このファイル(またはシートのリンク)をLINEで送ってください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>指名区分</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>名称</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>指名料(円)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>課金単位(何分ごと)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>バックの決め方</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>金額または率</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>円のときの単位</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>本指名</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>円</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>1接客ごと</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>場内指名</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="F9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>同伴</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>円</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>1接客ごと</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>ヘルプ</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>なし</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="n"/>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="n"/>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="7" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="n"/>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="n"/>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="7" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
-      <c r="F27" s="7" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="n"/>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
-      <c r="F28" s="7" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
-      <c r="F29" s="7" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="n"/>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="n"/>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
-      <c r="F31" s="7" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="n"/>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
-      <c r="F32" s="7" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="n"/>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="7" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="n"/>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
-      <c r="F34" s="7" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="n"/>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
-      <c r="F36" s="7" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="n"/>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
-      <c r="F37" s="7" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
-      <c r="F38" s="7" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="n"/>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="n"/>
-      <c r="B40" s="7" t="n"/>
-      <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
-      <c r="E40" s="7" t="n"/>
-      <c r="F40" s="7" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="n"/>
-      <c r="B41" s="7" t="n"/>
-      <c r="C41" s="7" t="n"/>
-      <c r="D41" s="7" t="n"/>
-      <c r="E41" s="7" t="n"/>
-      <c r="F41" s="7" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="B12:B41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="C12:C41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="D12:D41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
-      <formula1>"円,%,なし"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E12:E41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="0以上の数字で入力してください" type="decimal" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="F12:F41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="リストから選んでください" type="list">
-      <formula1>"1接客ごと,1時間ごと"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1832,7 +1392,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Move price sets and extension menu into the survey
Both tables are now filled in on the pricing section, so the LINE/Excel
kit drops the price sheet and keeps products and roster.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S7QD3LQaBHevrAWkRrJmwD
</commit_message>
<xml_diff>
--- a/templates/excel/初期設定_記入シート.xlsx
+++ b/templates/excel/初期設定_記入シート.xlsx
@@ -7,9 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="料金セット" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="商品メニュー" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="名簿" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="商品メニュー" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="名簿" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,513 +466,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D74"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>料金セット・延長メニュー</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>店舗名</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>※灰色の行は記入例です。消して上書きするか、下の空欄に書いてください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>※書き終わったら、このファイル(またはシートのリンク)をLINEで送ってください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>セット</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>セット名</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>時間(分)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>料金(円)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>延長(分)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>セット1</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>VIPセット</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="n"/>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="n"/>
-      <c r="B16" s="7" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="n"/>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="n"/>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="n"/>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="n"/>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="n"/>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="n"/>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="n"/>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="n"/>
-      <c r="B32" s="7" t="n"/>
-      <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="n"/>
-      <c r="B33" s="7" t="n"/>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="n"/>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="n"/>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="7" t="n"/>
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="n"/>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="n"/>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>延長</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>名前</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>時間(分)</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>料金(円)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>延長30分</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>延長60分</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="C44" s="6" t="n">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="n"/>
-      <c r="B45" s="7" t="n"/>
-      <c r="C45" s="7" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="7" t="n"/>
-      <c r="B46" s="7" t="n"/>
-      <c r="C46" s="7" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="n"/>
-      <c r="B47" s="7" t="n"/>
-      <c r="C47" s="7" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="7" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="n"/>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="7" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="n"/>
-      <c r="B50" s="7" t="n"/>
-      <c r="C50" s="7" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="n"/>
-      <c r="B51" s="7" t="n"/>
-      <c r="C51" s="7" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="n"/>
-      <c r="B52" s="7" t="n"/>
-      <c r="C52" s="7" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="7" t="n"/>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="7" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="n"/>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="7" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="7" t="n"/>
-      <c r="B55" s="7" t="n"/>
-      <c r="C55" s="7" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="n"/>
-      <c r="B56" s="7" t="n"/>
-      <c r="C56" s="7" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="7" t="n"/>
-      <c r="B57" s="7" t="n"/>
-      <c r="C57" s="7" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="7" t="n"/>
-      <c r="B58" s="7" t="n"/>
-      <c r="C58" s="7" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="7" t="n"/>
-      <c r="B59" s="7" t="n"/>
-      <c r="C59" s="7" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="7" t="n"/>
-      <c r="B60" s="7" t="n"/>
-      <c r="C60" s="7" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="7" t="n"/>
-      <c r="B61" s="7" t="n"/>
-      <c r="C61" s="7" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="7" t="n"/>
-      <c r="B62" s="7" t="n"/>
-      <c r="C62" s="7" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="7" t="n"/>
-      <c r="B63" s="7" t="n"/>
-      <c r="C63" s="7" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="7" t="n"/>
-      <c r="B64" s="7" t="n"/>
-      <c r="C64" s="7" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="7" t="n"/>
-      <c r="B65" s="7" t="n"/>
-      <c r="C65" s="7" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="7" t="n"/>
-      <c r="B66" s="7" t="n"/>
-      <c r="C66" s="7" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="7" t="n"/>
-      <c r="B67" s="7" t="n"/>
-      <c r="C67" s="7" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="7" t="n"/>
-      <c r="B68" s="7" t="n"/>
-      <c r="C68" s="7" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="7" t="n"/>
-      <c r="B69" s="7" t="n"/>
-      <c r="C69" s="7" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="7" t="n"/>
-      <c r="B70" s="7" t="n"/>
-      <c r="C70" s="7" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="7" t="n"/>
-      <c r="B71" s="7" t="n"/>
-      <c r="C71" s="7" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="7" t="n"/>
-      <c r="B72" s="7" t="n"/>
-      <c r="C72" s="7" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="7" t="n"/>
-      <c r="B73" s="7" t="n"/>
-      <c r="C73" s="7" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="7" t="n"/>
-      <c r="B74" s="7" t="n"/>
-      <c r="C74" s="7" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="B10:B39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="C10:C39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="D10:D39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="B45:B74" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation sqref="C45:C74" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="入力エラー" error="数字のみで入力してください(カンマ不要)" type="whole" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1392,7 +884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>